<commit_message>
refactor(memo-inquiry-90): apply 45-day structural architecture to 90-day inquiry memo and save as reference
</commit_message>
<xml_diff>
--- a/frontend/static/docs/ขอส่งใบติดตามทวงถาม_90_วัน_Rebuild_Thai.xlsx
+++ b/frontend/static/docs/ขอส่งใบติดตามทวงถาม_90_วัน_Rebuild_Thai.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="บันทึกข้อความ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบติดตามใบเบิก แผ่น 1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบติดตามใบเบิก แผ่น 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบติดตามใบเบิก_แผ่นที่1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบติดตามใบเบิก_แผ่นที่2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,17 +29,25 @@
     </font>
     <font>
       <name val="TH Sarabun PSK"/>
-      <b val="1"/>
-      <sz val="18"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="TH Sarabun PSK"/>
       <b val="1"/>
-      <sz val="12"/>
+      <sz val="24"/>
     </font>
     <font>
       <name val="TH Sarabun PSK"/>
-      <sz val="12"/>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="TH Sarabun PSK"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="TH Sarabun PSK"/>
+      <sz val="10.5"/>
     </font>
   </fonts>
   <fills count="2">
@@ -76,36 +84,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,133 +486,174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B4:E19"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="4">
-      <c r="C4" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>( สำเนาคู่ฉบับ )</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>บันทึกข้อความ</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="2" t="inlineStr">
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>ส่วนราชการ</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ป.พัน.๔ ร้อย.๒  ( โทร. ๓๑๑๙๓ )</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="2" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>ที่</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>กห ๐๔๘๓.๑.๔.๑ /       วันที่            มิ.ย. ๕๔</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>กห ๐๔๘๓.๑.๔.๑ /</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>วันที่</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>มิ.ย. ๕๔</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>เรื่อง</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>ขอส่งใบติดตามใบเบิก</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="2" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>เรียน</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>ผบ.ป.พัน.๔ ( ผ่าน ฝกบ. )</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>อ้างถึง</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>ระเบียบ ทบ. ว่าด้วยการส่งกำลัง สิ่งอุปกรณ์ ประเภท ๒ และ ๔ พ.ศ. ๒๕๓๔</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>สิ่งที่ส่งมาด้วย</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>- ใบติดตามใบเบิก   จำนวน ๒ ฉบับ</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>ใบติดตามใบเบิก   จำนวน ๒ ฉบับ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>ตามอ้างถึง ป.พัน.๔ ร้อย.๒ ขอส่งใบติดตามใบเบิก ตามห้วงระยะเวลาการเบิกเกิน ๙๐ วัน ซึ่งหน่วยได้ปฏิบัติตามระเบียบกองทัพบก ว่าด้วยการส่งกำลังสิ่งอุปกรณ์ ประเภท ๒ และ ๔ รายละเอียดตามสิ่งที่ส่งมาด้วย</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>จึงเรียนมาเพื่อกรุณาพิจารณาดำเนินการต่อไป</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="D18" s="4" t="inlineStr">
+    <row r="16">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>ร.อ.</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>(กฤติน  นราพงษ์)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="D19" s="6" t="inlineStr">
+    <row r="17">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>ผบ.ป.พัน.๔ ร้อย.๒</t>
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>จ.ส.อ.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>ร่าง/ตรวจ    มิ.ย. ๕๔</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>ส.อ. เสน่ห์ ฯ</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>พิมพ์      มิ.ย. ๕๔</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D19:E19"/>
+  <mergeCells count="3">
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B3:D3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -610,25 +665,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G21"/>
+  <dimension ref="A2:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>ใบติดตามใบเบิก</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>ทบ. ๔๐๐ - ๐๗๑
 แบบ ข การเบิกเกิน ๙๐ วัน</t>
@@ -636,334 +691,347 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ที่…………………………………………….</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>เรื่อง      ขอทราบผลการเบิก สป.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>ถึง   ป.พัน.๔</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>จาก   ป.พัน.๔ ร้อย.๒</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">        กรุณาดำเนินการตรวจสอบใบเบิกข้างล่างนี้ ซึ่งหน่วยได้ส่งใบเบิก และได้ติดตาม ครั้งที่ ๑ ไว้เรียบร้อยแล้ว</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>ลำดับ</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>รายการ สป.</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>หมายเลข สป.</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>ที่ใบเบิก ที่ทะเบียนหน่วยจ่าย</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>วันที่ส่งหรือวางใบเบิก</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>วันติดตามใบเบิกครั้งที่ ๒๐</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>หมายเหตุ (บันทึกโดยหน่วยจ่าย)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>๑.</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>ด้ามแส้ท่อนกกและปลาย</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>B ๙๗๒๔๒ - B ๑๙๗๒๔๒</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>๕๐ / ๔๗</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>๒๐ ก.พ. ๔๗</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>๒.</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>ไฟหลักเล็ง อันใกล้อันไกล</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>๑๒๙๐ – ๕๓๕ – ๗๖๒๙</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>๕๑ / ๔๗</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>๒๐ ก.พ. ๔๗</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>๓.</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>ซองหนังเครื่องตั้งมุมยิงประณีต</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>๑๒๙๐ – ๘๙๑ – ๙๙๙๙</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>๕๓ / ๔๗</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>๒๐ ก.พ. ๔๗</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr"/>
+      <c r="G13" s="11" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>๔.</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>ยางนอก</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>๒๖๑๐ – ๒๖๒ – ๘๘๑๖</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>๕๔ / ๔๗</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>๒๐ ก.พ. ๔๗</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr"/>
+      <c r="G14" s="11" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>๕.</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>แผ่นเป้าทดสอบ</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>๖๙๒๐ – ๗๑๔ – ๘๙๐๗</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>๗๐ / ๔๗</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>๑๗ มิ.ย. ๔๗</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr"/>
+      <c r="G15" s="11" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>๖.</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>น๊อตน้ำมันรับแรง</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>๔๗๓๐ – ๕๐๑ - ๘๔๙๕</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>๖๙ / ๔๗</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>๑๐ มิ.ย. ๔๗</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>๒ มิ.ย. ๕๒</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="E18" s="11" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>ผู้บังคับกองร้อย</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>ผู้ตรวจสอบ</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>ร.อ.</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>(กฤติน  นราพงษ์)</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>จ.ส.อ.</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>(ณัฐชัย  รักษาวงษ์)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="6" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>ผบ.ป.พัน.๔ ร้อย.๒</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>ส.หน.สย. ป.๔ พัน.๔ ร้อย.๒</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>มิ.ย. ๕๔</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>มิ.ย. ๕๔</t>
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          มิ.ย. ๕๔</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          มิ.ย. ๕๔</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>( พิมพ์ตามระเบียบกองทัพบกว่าด้วยการส่งกำลังสิ่งอุปกรณ์ ประเภท ๒ และ ๔ พ.ศ. ๒๕๓๔ )</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="E21:F21"/>
+  <mergeCells count="5">
+    <mergeCell ref="F21:G21"/>
     <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="F22:G22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -975,25 +1043,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G18"/>
+  <dimension ref="A2:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>ใบติดตามใบเบิก</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>ทบ. ๔๐๐ - ๐๗๑
 แบบ ข การเบิกเกิน ๙๐ วัน</t>
@@ -1001,235 +1069,248 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ที่…………………………………………….</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>เรื่อง      ขอทราบผลการเบิก สป.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>ถึง   ป.พัน.๔</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>จาก   ป.พัน.๔ ร้อย.๒</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">        กรุณาดำเนินการตรวจสอบใบเบิกข้างล่างนี้ ซึ่งหน่วยได้ส่งใบเบิก และได้ติดตาม ครั้งที่ ๑ ไว้เรียบร้อยแล้ว</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>ลำดับ</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>รายการ สป.</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>หมายเลข สป.</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>ที่ใบเบิก ที่ทะเบียนหน่วยจ่าย</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>วันที่ส่งหรือวางใบเบิก</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>วันติดตามใบเบิกครั้งที่ ๘</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>หมายเหตุ (บันทึกโดยหน่วยจ่าย)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>๑.</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>ยางใน</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>๒๓ / ๕๑</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>๑๓ มี.ค. ๕๑</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>๒.</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>ผ้าคลุมฐานกล้องเล็ง</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>๓๒๔๐ – ๐๐ – ๖๕๘ - ๒๘๒๒</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>๒๔ / ๕๑</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>๑๓ มี.ค. ๕๑</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>๓.</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>ผ้าคลุมฐานกล้องข้อศอก</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>๑๒๔๐ – ๐๐ – ๖๕๘ - ๒๘๒๓</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>๒๕ / ๕๑</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>๑๓ มี.ค. ๕๑</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>๑ มิ.ย. ๕๔</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="E15" s="11" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>ผู้บังคับกองร้อย</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>ผู้ตรวจสอบ</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>ร.อ.</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>(กฤติน  นราพงษ์)</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>จ.ส.อ.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>(ณัฐชัย  รักษาวงษ์)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>ผบ.ป.พัน.๔ ร้อย.๒</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>ส.หน.สย. ป.๔ พัน.๔ ร้อย.๒</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>มิ.ย. ๕๔</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>มิ.ย. ๕๔</t>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          มิ.ย. ๕๔</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          มิ.ย. ๕๔</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>( พิมพ์ตามระเบียบกองทัพบกว่าด้วยการส่งกำลังสิ่งอุปกรณ์ ประเภท ๒ และ ๔ พ.ศ. ๒๕๓๔ )</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F18:G18"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>